<commit_message>
chore: publish latest code
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -474,13 +474,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9128.969999999999</v>
+        <v>9216</v>
       </c>
       <c r="F2" t="n">
-        <v>8135.8</v>
+        <v>8009.8</v>
       </c>
       <c r="G2" t="n">
-        <v>993.17</v>
+        <v>1206.2</v>
       </c>
     </row>
   </sheetData>
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4016.97</v>
+        <v>4496</v>
       </c>
       <c r="C2" t="n">
-        <v>5429.8</v>
+        <v>5368.8</v>
       </c>
       <c r="D2" t="n">
-        <v>-1412.83</v>
+        <v>-872.8</v>
       </c>
       <c r="E2" t="n">
-        <v>4016.97</v>
+        <v>4496</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -558,88 +558,88 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>135.17</v>
+        <v>119.41</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1744</v>
+        <v>1632</v>
       </c>
       <c r="C3" t="n">
-        <v>1110</v>
+        <v>1457</v>
       </c>
       <c r="D3" t="n">
-        <v>634</v>
+        <v>175</v>
       </c>
       <c r="E3" t="n">
-        <v>1744</v>
+        <v>1632</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>63.65</v>
+        <v>89.28</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1632</v>
+        <v>1496</v>
       </c>
       <c r="C4" t="n">
-        <v>1481</v>
+        <v>112</v>
       </c>
       <c r="D4" t="n">
-        <v>151</v>
+        <v>1384</v>
       </c>
       <c r="E4" t="n">
-        <v>1632</v>
+        <v>1496</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>90.75</v>
+        <v>7.49</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1496</v>
+        <v>1352</v>
       </c>
       <c r="C5" t="n">
-        <v>112</v>
+        <v>1069</v>
       </c>
       <c r="D5" t="n">
-        <v>1384</v>
+        <v>283</v>
       </c>
       <c r="E5" t="n">
-        <v>1496</v>
+        <v>1352</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>7.49</v>
+        <v>79.06999999999999</v>
       </c>
     </row>
     <row r="6">
@@ -658,7 +658,7 @@
         <v>237</v>
       </c>
       <c r="E6" t="n">
-        <v>181.46</v>
+        <v>187.32</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update latest reports, scripts, and tests
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -477,10 +477,10 @@
         <v>9216</v>
       </c>
       <c r="F2" t="n">
-        <v>8009.8</v>
+        <v>8712.799999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>1206.2</v>
+        <v>503.2</v>
       </c>
     </row>
   </sheetData>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,10 +544,10 @@
         <v>4496</v>
       </c>
       <c r="C2" t="n">
-        <v>5368.8</v>
+        <v>5228.8</v>
       </c>
       <c r="D2" t="n">
-        <v>-872.8</v>
+        <v>-732.8</v>
       </c>
       <c r="E2" t="n">
         <v>4496</v>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>119.41</v>
+        <v>116.3</v>
       </c>
     </row>
     <row r="3">
@@ -658,7 +658,7 @@
         <v>237</v>
       </c>
       <c r="E6" t="n">
-        <v>187.32</v>
+        <v>193.17</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -667,6 +667,52 @@
       </c>
       <c r="G6" t="n">
         <v>1.25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WOM</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>843</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-843</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync: reports, scripts, tests, docs; ignore large DB files
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -474,13 +474,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>8192</v>
+        <v>9576</v>
       </c>
       <c r="F2" t="n">
-        <v>8680.799999999999</v>
+        <v>8696.799999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>-488.8</v>
+        <v>879.2</v>
       </c>
     </row>
   </sheetData>
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3472</v>
+        <v>4856</v>
       </c>
       <c r="C2" t="n">
-        <v>5196.8</v>
+        <v>5212.8</v>
       </c>
       <c r="D2" t="n">
-        <v>-1724.8</v>
+        <v>-356.8</v>
       </c>
       <c r="E2" t="n">
-        <v>3472</v>
+        <v>4856</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>149.68</v>
+        <v>107.35</v>
       </c>
     </row>
     <row r="3">
@@ -658,7 +658,7 @@
         <v>237</v>
       </c>
       <c r="E6" t="n">
-        <v>216.59</v>
+        <v>222.44</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Replace repository contents with local project snapshot
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -474,13 +474,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9576</v>
+        <v>8582.67</v>
       </c>
       <c r="F2" t="n">
-        <v>8696.799999999999</v>
+        <v>46484.68</v>
       </c>
       <c r="G2" t="n">
-        <v>879.2</v>
+        <v>-37902.01</v>
       </c>
     </row>
   </sheetData>
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4856</v>
+        <v>3654.67</v>
       </c>
       <c r="C2" t="n">
-        <v>5212.8</v>
+        <v>32264.76</v>
       </c>
       <c r="D2" t="n">
-        <v>-356.8</v>
+        <v>-28610.09</v>
       </c>
       <c r="E2" t="n">
-        <v>4856</v>
+        <v>3654.67</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -558,61 +558,61 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>107.35</v>
+        <v>882.84</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1632</v>
+        <v>1897</v>
       </c>
       <c r="C3" t="n">
-        <v>1457</v>
+        <v>977</v>
       </c>
       <c r="D3" t="n">
-        <v>175</v>
+        <v>920</v>
       </c>
       <c r="E3" t="n">
-        <v>1632</v>
+        <v>1897</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>89.28</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1496</v>
+        <v>1688</v>
       </c>
       <c r="C4" t="n">
-        <v>112</v>
+        <v>5528</v>
       </c>
       <c r="D4" t="n">
-        <v>1384</v>
+        <v>-3840</v>
       </c>
       <c r="E4" t="n">
-        <v>1496</v>
+        <v>1688</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>7.49</v>
+        <v>327.49</v>
       </c>
     </row>
     <row r="5">
@@ -622,16 +622,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1352</v>
+        <v>1053</v>
       </c>
       <c r="C5" t="n">
-        <v>1069</v>
+        <v>7071.92</v>
       </c>
       <c r="D5" t="n">
-        <v>283</v>
+        <v>-6018.92</v>
       </c>
       <c r="E5" t="n">
-        <v>1352</v>
+        <v>1053</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>79.06999999999999</v>
+        <v>671.6</v>
       </c>
     </row>
     <row r="6">
@@ -649,16 +649,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>294</v>
       </c>
       <c r="D6" t="n">
-        <v>237</v>
+        <v>-44</v>
       </c>
       <c r="E6" t="n">
-        <v>222.44</v>
+        <v>243.9</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -666,46 +666,46 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1.25</v>
+        <v>117.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WOM</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C7" t="n">
-        <v>843</v>
+        <v>87</v>
       </c>
       <c r="D7" t="n">
-        <v>-843</v>
+        <v>-47</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>217.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>WOM</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>262</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>-262</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat: sync dashboard refresh and db-backed reports
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -474,13 +474,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>8582.67</v>
+        <v>9696</v>
       </c>
       <c r="F2" t="n">
-        <v>46484.68</v>
+        <v>7771.13</v>
       </c>
       <c r="G2" t="n">
-        <v>-37902.01</v>
+        <v>1924.87</v>
       </c>
     </row>
   </sheetData>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3654.67</v>
+        <v>4336</v>
       </c>
       <c r="C2" t="n">
-        <v>32264.76</v>
+        <v>5230.13</v>
       </c>
       <c r="D2" t="n">
-        <v>-28610.09</v>
+        <v>-894.13</v>
       </c>
       <c r="E2" t="n">
-        <v>3654.67</v>
+        <v>4336</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -558,61 +558,61 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>882.84</v>
+        <v>120.62</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1897</v>
+        <v>1752</v>
       </c>
       <c r="C3" t="n">
-        <v>977</v>
+        <v>1463</v>
       </c>
       <c r="D3" t="n">
-        <v>920</v>
+        <v>289</v>
       </c>
       <c r="E3" t="n">
-        <v>1897</v>
+        <v>1752</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>51.5</v>
+        <v>83.5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1688</v>
+        <v>1496</v>
       </c>
       <c r="C4" t="n">
-        <v>5528</v>
+        <v>104</v>
       </c>
       <c r="D4" t="n">
-        <v>-3840</v>
+        <v>1392</v>
       </c>
       <c r="E4" t="n">
-        <v>1688</v>
+        <v>1496</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>327.49</v>
+        <v>6.95</v>
       </c>
     </row>
     <row r="5">
@@ -622,16 +622,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1053</v>
+        <v>1352</v>
       </c>
       <c r="C5" t="n">
-        <v>7071.92</v>
+        <v>971</v>
       </c>
       <c r="D5" t="n">
-        <v>-6018.92</v>
+        <v>381</v>
       </c>
       <c r="E5" t="n">
-        <v>1053</v>
+        <v>1352</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -639,57 +639,61 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>671.6</v>
+        <v>71.81999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ODL</t>
+          <t>SUBS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>250</v>
+        <v>520</v>
       </c>
       <c r="C6" t="n">
-        <v>294</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-44</v>
+        <v>520</v>
       </c>
       <c r="E6" t="n">
-        <v>243.9</v>
+        <v>520</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>117.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ODL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>240</v>
       </c>
       <c r="C7" t="n">
-        <v>87</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>-47</v>
+        <v>237</v>
       </c>
       <c r="E7" t="n">
-        <v>40</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>240</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
       <c r="G7" t="n">
-        <v>217.5</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="8">
@@ -702,16 +706,62 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>-262</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>OAM</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CRM</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: refresh report server and leave outputs
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -462,25 +462,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>9696</v>
+        <v>10488</v>
       </c>
       <c r="F2" t="n">
-        <v>7771.13</v>
+        <v>7833.13</v>
       </c>
       <c r="G2" t="n">
-        <v>1924.87</v>
+        <v>2654.87</v>
       </c>
     </row>
   </sheetData>
@@ -541,24 +541,24 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4336</v>
+        <v>6704</v>
       </c>
       <c r="C2" t="n">
-        <v>5230.13</v>
+        <v>5238.13</v>
       </c>
       <c r="D2" t="n">
-        <v>-894.13</v>
+        <v>1465.87</v>
       </c>
       <c r="E2" t="n">
-        <v>4336</v>
+        <v>6704</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-02-06</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>120.62</v>
+        <v>78.13</v>
       </c>
     </row>
     <row r="3">
@@ -568,24 +568,24 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1752</v>
+        <v>1712</v>
       </c>
       <c r="C3" t="n">
-        <v>1463</v>
+        <v>1455</v>
       </c>
       <c r="D3" t="n">
-        <v>289</v>
+        <v>257</v>
       </c>
       <c r="E3" t="n">
-        <v>1752</v>
+        <v>1712</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>83.5</v>
+        <v>84.98999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -595,105 +595,105 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1496</v>
+        <v>1192</v>
       </c>
       <c r="C4" t="n">
-        <v>104</v>
+        <v>165.5</v>
       </c>
       <c r="D4" t="n">
-        <v>1392</v>
+        <v>1026.5</v>
       </c>
       <c r="E4" t="n">
-        <v>1496</v>
+        <v>1192</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>6.95</v>
+        <v>13.88</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>SUBS</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1352</v>
+        <v>520</v>
       </c>
       <c r="C5" t="n">
-        <v>971</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>381</v>
+        <v>520</v>
       </c>
       <c r="E5" t="n">
-        <v>1352</v>
+        <v>520</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>71.81999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SUBS</t>
+          <t>ODL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>520</v>
+        <v>240</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D6" t="n">
-        <v>520</v>
+        <v>237</v>
       </c>
       <c r="E6" t="n">
-        <v>520</v>
+        <v>240</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ODL</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>971.5</v>
       </c>
       <c r="D7" t="n">
-        <v>237</v>
+        <v>-851.5</v>
       </c>
       <c r="E7" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1.25</v>
+        <v>809.58</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Sync reports, RMI gantt, tests, and docs; stop tracking .env; expand gitignore for local assets
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -467,20 +467,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>10488</v>
+        <v>11340</v>
       </c>
       <c r="F2" t="n">
-        <v>7833.13</v>
+        <v>7915.18</v>
       </c>
       <c r="G2" t="n">
-        <v>2654.87</v>
+        <v>3424.82</v>
       </c>
     </row>
   </sheetData>
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6704</v>
+        <v>3913.6</v>
       </c>
       <c r="C2" t="n">
-        <v>5238.13</v>
+        <v>5276.68</v>
       </c>
       <c r="D2" t="n">
-        <v>1465.87</v>
+        <v>-1363.08</v>
       </c>
       <c r="E2" t="n">
-        <v>6704</v>
+        <v>3913.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -558,34 +558,34 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>78.13</v>
+        <v>134.83</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1712</v>
+        <v>3496</v>
       </c>
       <c r="C3" t="n">
-        <v>1455</v>
+        <v>1011.5</v>
       </c>
       <c r="D3" t="n">
-        <v>257</v>
+        <v>2484.5</v>
       </c>
       <c r="E3" t="n">
-        <v>1712</v>
+        <v>3496</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>84.98999999999999</v>
+        <v>28.93</v>
       </c>
     </row>
     <row r="4">
@@ -595,16 +595,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1192</v>
+        <v>1832</v>
       </c>
       <c r="C4" t="n">
-        <v>165.5</v>
+        <v>144</v>
       </c>
       <c r="D4" t="n">
-        <v>1026.5</v>
+        <v>1688</v>
       </c>
       <c r="E4" t="n">
-        <v>1192</v>
+        <v>1832</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -612,88 +612,88 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>13.88</v>
+        <v>7.86</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SUBS</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>520</v>
+        <v>1338.4</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1480</v>
       </c>
       <c r="D5" t="n">
-        <v>520</v>
+        <v>-141.6</v>
       </c>
       <c r="E5" t="n">
-        <v>520</v>
+        <v>1338.4</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>110.58</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ODL</t>
+          <t>SUBS</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>240</v>
+        <v>520</v>
       </c>
       <c r="C6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>237</v>
+        <v>520</v>
       </c>
       <c r="E6" t="n">
-        <v>240</v>
+        <v>520</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-13</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>ODL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="C7" t="n">
-        <v>971.5</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>-851.5</v>
+        <v>237</v>
       </c>
       <c r="E7" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-13</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>809.58</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
Sync reports, docs, Azure App Service wiring, and CI workflow
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -462,25 +462,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>11496</v>
+        <v>10021.6</v>
       </c>
       <c r="F2" t="n">
         <v>7928.68</v>
       </c>
       <c r="G2" t="n">
-        <v>3567.32</v>
+        <v>2092.92</v>
       </c>
     </row>
   </sheetData>
@@ -541,24 +541,24 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4153.6</v>
+        <v>3735.2</v>
       </c>
       <c r="C2" t="n">
         <v>5278.18</v>
       </c>
       <c r="D2" t="n">
-        <v>-1124.58</v>
+        <v>-1542.98</v>
       </c>
       <c r="E2" t="n">
-        <v>4153.6</v>
+        <v>3735.2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>127.07</v>
+        <v>141.31</v>
       </c>
     </row>
     <row r="3">
@@ -568,24 +568,24 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3496</v>
+        <v>3376</v>
       </c>
       <c r="C3" t="n">
         <v>1015.5</v>
       </c>
       <c r="D3" t="n">
-        <v>2480.5</v>
+        <v>2360.5</v>
       </c>
       <c r="E3" t="n">
-        <v>3496</v>
+        <v>3376</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>29.05</v>
+        <v>30.08</v>
       </c>
     </row>
     <row r="4">
@@ -595,121 +595,117 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1832</v>
+        <v>1664</v>
       </c>
       <c r="C4" t="n">
         <v>144</v>
       </c>
       <c r="D4" t="n">
-        <v>1688</v>
+        <v>1520</v>
       </c>
       <c r="E4" t="n">
-        <v>1832</v>
+        <v>1664</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>7.86</v>
+        <v>8.65</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>WOM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1254.4</v>
+        <v>744</v>
       </c>
       <c r="C5" t="n">
-        <v>1488</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>-233.6</v>
+        <v>744</v>
       </c>
       <c r="E5" t="n">
-        <v>1254.4</v>
+        <v>694.4</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>118.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SUBS</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>520</v>
+        <v>502.4</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1488</v>
       </c>
       <c r="D6" t="n">
-        <v>520</v>
+        <v>-985.6</v>
       </c>
       <c r="E6" t="n">
-        <v>520</v>
+        <v>502.4</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-06</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>296.18</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ODL</t>
+          <t>SUBS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>240</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
-        <v>237</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>240</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WOM</t>
+          <t>ODL</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Sync local changes: navigation, report HTML, generated data, and module updates to match localhost
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -477,10 +477,10 @@
         <v>10021.6</v>
       </c>
       <c r="F2" t="n">
-        <v>7928.68</v>
+        <v>7925.63</v>
       </c>
       <c r="G2" t="n">
-        <v>2092.92</v>
+        <v>2095.97</v>
       </c>
     </row>
   </sheetData>
@@ -544,10 +544,10 @@
         <v>3735.2</v>
       </c>
       <c r="C2" t="n">
-        <v>5278.18</v>
+        <v>5275.13</v>
       </c>
       <c r="D2" t="n">
-        <v>-1542.98</v>
+        <v>-1539.93</v>
       </c>
       <c r="E2" t="n">
         <v>3735.2</v>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>141.31</v>
+        <v>141.23</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Update report server and generated reports
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -474,13 +474,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>10021.6</v>
+        <v>12808.8</v>
       </c>
       <c r="F2" t="n">
-        <v>7925.63</v>
+        <v>8183.63</v>
       </c>
       <c r="G2" t="n">
-        <v>2095.97</v>
+        <v>4625.17</v>
       </c>
     </row>
   </sheetData>
@@ -541,16 +541,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3735.2</v>
+        <v>5719.2</v>
       </c>
       <c r="C2" t="n">
-        <v>5275.13</v>
+        <v>5291.13</v>
       </c>
       <c r="D2" t="n">
-        <v>-1539.93</v>
+        <v>428.07</v>
       </c>
       <c r="E2" t="n">
-        <v>3735.2</v>
+        <v>5719.2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -558,7 +558,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>141.23</v>
+        <v>92.52</v>
       </c>
     </row>
     <row r="3">
@@ -568,24 +568,24 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3376</v>
+        <v>3472</v>
       </c>
       <c r="C3" t="n">
-        <v>1015.5</v>
+        <v>1029.5</v>
       </c>
       <c r="D3" t="n">
-        <v>2360.5</v>
+        <v>2442.5</v>
       </c>
       <c r="E3" t="n">
-        <v>3376</v>
+        <v>3472</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>30.08</v>
+        <v>29.65</v>
       </c>
     </row>
     <row r="4">
@@ -618,55 +618,55 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WOM</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>744</v>
+        <v>1209.6</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1700</v>
       </c>
       <c r="D5" t="n">
-        <v>744</v>
+        <v>-490.4</v>
       </c>
       <c r="E5" t="n">
-        <v>694.4</v>
+        <v>1209.6</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>140.54</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>WOM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>502.4</v>
+        <v>744</v>
       </c>
       <c r="C6" t="n">
-        <v>1488</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>-985.6</v>
+        <v>744</v>
       </c>
       <c r="E6" t="n">
-        <v>502.4</v>
+        <v>727.47</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>296.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -702,10 +702,10 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="D8" t="n">
-        <v>-3</v>
+        <v>-19</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: sync latest local changes to main
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -477,10 +477,10 @@
         <v>12808.8</v>
       </c>
       <c r="F2" t="n">
-        <v>8183.63</v>
+        <v>8177.63</v>
       </c>
       <c r="G2" t="n">
-        <v>4625.17</v>
+        <v>4631.17</v>
       </c>
     </row>
   </sheetData>
@@ -625,10 +625,10 @@
         <v>1209.6</v>
       </c>
       <c r="C5" t="n">
-        <v>1700</v>
+        <v>1694</v>
       </c>
       <c r="D5" t="n">
-        <v>-490.4</v>
+        <v>-484.4</v>
       </c>
       <c r="E5" t="n">
         <v>1209.6</v>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>140.54</v>
+        <v>140.05</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
fix(epics-planner): add Jira URL input to sync modal for TMP epics
TMP epics created in the Epics Planner had no way to provide a Jira URL
during sync, causing a 400 BAD REQUEST. The sync modal now includes a
required Jira URL field that is pre-filled from the row's existing URL.
On sync, the backend also auto-promotes TMP keys to real Jira keys and
sets the project_key for ORPHAN rows.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -462,25 +462,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>12808.8</v>
+        <v>10776</v>
       </c>
       <c r="F2" t="n">
-        <v>8177.63</v>
+        <v>8661.23</v>
       </c>
       <c r="G2" t="n">
-        <v>4631.17</v>
+        <v>2114.77</v>
       </c>
     </row>
   </sheetData>
@@ -541,24 +541,24 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5719.2</v>
+        <v>4958.4</v>
       </c>
       <c r="C2" t="n">
-        <v>5291.13</v>
+        <v>5663.13</v>
       </c>
       <c r="D2" t="n">
-        <v>428.07</v>
+        <v>-704.73</v>
       </c>
       <c r="E2" t="n">
-        <v>5719.2</v>
+        <v>4958.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>92.52</v>
+        <v>114.21</v>
       </c>
     </row>
     <row r="3">
@@ -568,16 +568,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3472</v>
+        <v>3688</v>
       </c>
       <c r="C3" t="n">
-        <v>1029.5</v>
+        <v>1055.5</v>
       </c>
       <c r="D3" t="n">
-        <v>2442.5</v>
+        <v>2632.5</v>
       </c>
       <c r="E3" t="n">
-        <v>3472</v>
+        <v>3688</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -585,61 +585,61 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>29.65</v>
+        <v>28.62</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MN</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1664</v>
+        <v>1297.6</v>
       </c>
       <c r="C4" t="n">
-        <v>144</v>
+        <v>1730</v>
       </c>
       <c r="D4" t="n">
-        <v>1520</v>
+        <v>-432.4</v>
       </c>
       <c r="E4" t="n">
-        <v>1664</v>
+        <v>1297.6</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>8.65</v>
+        <v>133.32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>MN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1209.6</v>
+        <v>832</v>
       </c>
       <c r="C5" t="n">
-        <v>1694</v>
+        <v>152</v>
       </c>
       <c r="D5" t="n">
-        <v>-484.4</v>
+        <v>680</v>
       </c>
       <c r="E5" t="n">
-        <v>1209.6</v>
+        <v>832</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>140.05</v>
+        <v>18.27</v>
       </c>
     </row>
     <row r="6">
@@ -649,22 +649,18 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>744</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>744</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>744</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>0</v>
       </c>
@@ -702,15 +698,19 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>19</v>
+        <v>36.6</v>
       </c>
       <c r="D8" t="n">
-        <v>-19</v>
+        <v>-36.6</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
@@ -725,10 +725,10 @@
         <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>-24</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Push today's report, epic explorer, and RnD muscle updates
Includes epic explorer service/report, RnD muscle utilization API + docs,
RLT leave report, synced report_html outputs, shared-nav, and related tests.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rnd_data_story_dataset.xlsx
+++ b/rnd_data_story_dataset.xlsx
@@ -462,25 +462,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>10776</v>
+        <v>8226.4</v>
       </c>
       <c r="F2" t="n">
-        <v>8661.23</v>
+        <v>9038.58</v>
       </c>
       <c r="G2" t="n">
-        <v>2114.77</v>
+        <v>-812.1799999999999</v>
       </c>
     </row>
   </sheetData>
@@ -541,78 +541,78 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4958.4</v>
+        <v>5254.4</v>
       </c>
       <c r="C2" t="n">
-        <v>5663.13</v>
+        <v>5987.13</v>
       </c>
       <c r="D2" t="n">
-        <v>-704.73</v>
+        <v>-732.73</v>
       </c>
       <c r="E2" t="n">
-        <v>4958.4</v>
+        <v>5254.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>114.21</v>
+        <v>113.95</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FF</t>
+          <t>DIGITALLOG</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3688</v>
+        <v>1612</v>
       </c>
       <c r="C3" t="n">
-        <v>1055.5</v>
+        <v>1747.6</v>
       </c>
       <c r="D3" t="n">
-        <v>2632.5</v>
+        <v>-135.6</v>
       </c>
       <c r="E3" t="n">
-        <v>3688</v>
+        <v>1612</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>28.62</v>
+        <v>108.41</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DIGITALLOG</t>
+          <t>FF</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1297.6</v>
+        <v>1120</v>
       </c>
       <c r="C4" t="n">
-        <v>1730</v>
+        <v>1071.5</v>
       </c>
       <c r="D4" t="n">
-        <v>-432.4</v>
+        <v>48.5</v>
       </c>
       <c r="E4" t="n">
-        <v>1297.6</v>
+        <v>1120</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>133.32</v>
+        <v>95.67</v>
       </c>
     </row>
     <row r="5">
@@ -622,24 +622,24 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>832</v>
+        <v>240</v>
       </c>
       <c r="C5" t="n">
         <v>152</v>
       </c>
       <c r="D5" t="n">
-        <v>680</v>
+        <v>88</v>
       </c>
       <c r="E5" t="n">
-        <v>832</v>
+        <v>240</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>18.27</v>
+        <v>63.33</v>
       </c>
     </row>
     <row r="6">
@@ -698,17 +698,17 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>36.6</v>
+        <v>56.35</v>
       </c>
       <c r="D8" t="n">
-        <v>-36.6</v>
+        <v>-56.35</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="G8" t="n">

</xml_diff>